<commit_message>
Added mean temperature data, calculated as the average of max and min temperatures (as recommended by easyclimate, see https://verughub.github.io/easyclimate/articles/climatic-indices.html)
</commit_message>
<xml_diff>
--- a/02_clean_data/02_03_site_means.xlsx
+++ b/02_clean_data/02_03_site_means.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>pair_id</t>
   </si>
@@ -63,6 +63,18 @@
   </si>
   <si>
     <t>T_min_min</t>
+  </si>
+  <si>
+    <t>T_mean_mean</t>
+  </si>
+  <si>
+    <t>T_mean_sd</t>
+  </si>
+  <si>
+    <t>T_mean_max</t>
+  </si>
+  <si>
+    <t>T_mean_min</t>
   </si>
   <si>
     <t>spei12_mean</t>
@@ -241,13 +253,25 @@
       <c r="X1" t="s">
         <v>22</v>
       </c>
+      <c r="Y1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C2" t="n">
         <v>1507.0194</v>
@@ -298,30 +322,42 @@
         <v>-0.00882191780821919</v>
       </c>
       <c r="S2" t="n">
+        <v>8.47818209320346</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.932967178795355</v>
+      </c>
+      <c r="U2" t="n">
+        <v>11.141465753424665</v>
+      </c>
+      <c r="V2" t="n">
+        <v>6.14680821917809</v>
+      </c>
+      <c r="W2" t="n">
         <v>-0.09592004850180864</v>
       </c>
-      <c r="T2" t="n">
+      <c r="X2" t="n">
         <v>1.0599272807536326</v>
       </c>
-      <c r="U2" t="n">
+      <c r="Y2" t="n">
         <v>2.54410123825073</v>
       </c>
-      <c r="V2" t="n">
+      <c r="Z2" t="n">
         <v>-3.15736532211304</v>
       </c>
-      <c r="W2" t="n">
+      <c r="AA2" t="n">
         <v>-0.10868326613552626</v>
       </c>
-      <c r="X2" t="n">
+      <c r="AB2" t="n">
         <v>-0.12143659156284115</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C3" t="n">
         <v>1078.5381818181818</v>
@@ -372,30 +408,42 @@
         <v>0.542356164383562</v>
       </c>
       <c r="S3" t="n">
+        <v>9.060242822619385</v>
+      </c>
+      <c r="T3" t="n">
+        <v>1.113513345139292</v>
+      </c>
+      <c r="U3" t="n">
+        <v>12.676890410958926</v>
+      </c>
+      <c r="V3" t="n">
+        <v>6.617849315068481</v>
+      </c>
+      <c r="W3" t="n">
         <v>-0.05350274368407422</v>
       </c>
-      <c r="T3" t="n">
+      <c r="X3" t="n">
         <v>1.0201379142418494</v>
       </c>
-      <c r="U3" t="n">
+      <c r="Y3" t="n">
         <v>2.50756478309631</v>
       </c>
-      <c r="V3" t="n">
+      <c r="Z3" t="n">
         <v>-2.84572267532349</v>
       </c>
-      <c r="W3" t="n">
+      <c r="AA3" t="n">
         <v>-0.05761140134046082</v>
       </c>
-      <c r="X3" t="n">
+      <c r="AB3" t="n">
         <v>-0.060883716173021143</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C4" t="n">
         <v>732.5802941176471</v>
@@ -446,30 +494,42 @@
         <v>6.58945355191257</v>
       </c>
       <c r="S4" t="n">
+        <v>14.102289767741015</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.9247332909939024</v>
+      </c>
+      <c r="U4" t="n">
+        <v>16.83294520547945</v>
+      </c>
+      <c r="V4" t="n">
+        <v>11.901010928961755</v>
+      </c>
+      <c r="W4" t="n">
         <v>-0.20298888804874785</v>
       </c>
-      <c r="T4" t="n">
+      <c r="X4" t="n">
         <v>0.9975652085112111</v>
       </c>
-      <c r="U4" t="n">
+      <c r="Y4" t="n">
         <v>2.4429292678833</v>
       </c>
-      <c r="V4" t="n">
+      <c r="Z4" t="n">
         <v>-2.39087724685669</v>
       </c>
-      <c r="W4" t="n">
+      <c r="AA4" t="n">
         <v>-0.23940388196612583</v>
       </c>
-      <c r="X4" t="n">
+      <c r="AB4" t="n">
         <v>-0.26672997342177185</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C5" t="n">
         <v>1408.6835384615385</v>
@@ -520,30 +580,42 @@
         <v>2.86494535519126</v>
       </c>
       <c r="S5" t="n">
+        <v>10.092604736501308</v>
+      </c>
+      <c r="T5" t="n">
+        <v>1.0497434490303703</v>
+      </c>
+      <c r="U5" t="n">
+        <v>13.45606849315068</v>
+      </c>
+      <c r="V5" t="n">
+        <v>7.169904371584715</v>
+      </c>
+      <c r="W5" t="n">
         <v>-0.1448657144471843</v>
       </c>
-      <c r="T5" t="n">
+      <c r="X5" t="n">
         <v>1.0481252591437646</v>
       </c>
-      <c r="U5" t="n">
+      <c r="Y5" t="n">
         <v>2.4408233165741</v>
       </c>
-      <c r="V5" t="n">
+      <c r="Z5" t="n">
         <v>-2.50002098083496</v>
       </c>
-      <c r="W5" t="n">
+      <c r="AA5" t="n">
         <v>-0.17640545240473335</v>
       </c>
-      <c r="X5" t="n">
+      <c r="AB5" t="n">
         <v>-0.19986586218159946</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C6" t="n">
         <v>755.4</v>
@@ -594,30 +666,42 @@
         <v>2.79572602739726</v>
       </c>
       <c r="S6" t="n">
+        <v>10.880090049984261</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.8491495324793265</v>
+      </c>
+      <c r="U6" t="n">
+        <v>13.93184931506848</v>
+      </c>
+      <c r="V6" t="n">
+        <v>8.961452054794531</v>
+      </c>
+      <c r="W6" t="n">
         <v>-0.08686802402732056</v>
       </c>
-      <c r="T6" t="n">
+      <c r="X6" t="n">
         <v>1.0098490121063766</v>
       </c>
-      <c r="U6" t="n">
+      <c r="Y6" t="n">
         <v>2.50756478309631</v>
       </c>
-      <c r="V6" t="n">
+      <c r="Z6" t="n">
         <v>-2.84572267532349</v>
       </c>
-      <c r="W6" t="n">
+      <c r="AA6" t="n">
         <v>-0.09679541325224394</v>
       </c>
-      <c r="X6" t="n">
+      <c r="AB6" t="n">
         <v>-0.10504481346045702</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C7" t="n">
         <v>1029.3755</v>
@@ -668,30 +752,42 @@
         <v>0.166684931506849</v>
       </c>
       <c r="S7" t="n">
+        <v>9.62122193843632</v>
+      </c>
+      <c r="T7" t="n">
+        <v>1.3667012145147903</v>
+      </c>
+      <c r="U7" t="n">
+        <v>13.41090410958902</v>
+      </c>
+      <c r="V7" t="n">
+        <v>6.609383561643824</v>
+      </c>
+      <c r="W7" t="n">
         <v>-0.05350274368407421</v>
       </c>
-      <c r="T7" t="n">
+      <c r="X7" t="n">
         <v>1.020133562294022</v>
       </c>
-      <c r="U7" t="n">
+      <c r="Y7" t="n">
         <v>2.50756478309631</v>
       </c>
-      <c r="V7" t="n">
+      <c r="Z7" t="n">
         <v>-2.84572267532349</v>
       </c>
-      <c r="W7" t="n">
+      <c r="AA7" t="n">
         <v>-0.057611401340460826</v>
       </c>
-      <c r="X7" t="n">
+      <c r="AB7" t="n">
         <v>-0.060883716173021143</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C8" t="n">
         <v>1400.5452500000001</v>
@@ -742,21 +838,33 @@
         <v>1.10230136986301</v>
       </c>
       <c r="S8" t="n">
+        <v>9.345769688939544</v>
+      </c>
+      <c r="T8" t="n">
+        <v>1.0138249305900522</v>
+      </c>
+      <c r="U8" t="n">
+        <v>12.40532876712327</v>
+      </c>
+      <c r="V8" t="n">
+        <v>6.7530601092896205</v>
+      </c>
+      <c r="W8" t="n">
         <v>-0.0021631405969371803</v>
       </c>
-      <c r="T8" t="n">
+      <c r="X8" t="n">
         <v>1.0836751750776399</v>
       </c>
-      <c r="U8" t="n">
+      <c r="Y8" t="n">
         <v>2.66420936584473</v>
       </c>
-      <c r="V8" t="n">
+      <c r="Z8" t="n">
         <v>-3.55342841148376</v>
       </c>
-      <c r="W8" t="n">
+      <c r="AA8" t="n">
         <v>0.006734416437301773</v>
       </c>
-      <c r="X8" t="n">
+      <c r="AB8" t="n">
         <v>0.011372408274952402</v>
       </c>
     </row>

</xml_diff>